<commit_message>
Documentation v1.1: reflect security/performance/SEO hardening
- New 3.4 Performance measures section (LCP fetchPriority, asset caching,
  lazy loading, zero-JS banner animation)
- Security posture: per-IP rate limits on all email routes documented
- SEO: robots /api/ exclusion + X-Robots-Tag noted
- Limitations: rate-limiting gap replaced with the per-instance caveat
- Services spreadsheet: API Routes sheet carries each route's rate limit

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018A5h36uWK4kcZoHCyNmetT
</commit_message>
<xml_diff>
--- a/docs/dareomotosho-services.xlsx
+++ b/docs/dareomotosho-services.xlsx
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>422 'invalid from' = sender not on the verified domain or malformed env var (now sanitized by lib/email.ts safeSender).</t>
+          <t>Rate limit: 5 requests / 10 min per IP. 422 'invalid from' = sender not on the verified domain or malformed env var (now sanitized by lib/email.ts safeSender).</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>GET reports key presence, audience list, and the ID in use. 409 (already subscribed) counts as success.</t>
+          <t>Rate limit: 8 requests / 10 min per IP (POST). GET reports key presence, audience list, and the ID in use. 409 (already subscribed) counts as success.</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Reply-To set as a raw header to avoid the reply_to/replyTo API naming variance. Honeypot hits return fake success.</t>
+          <t>Rate limits: POST 5 / 10 min per IP; ?send=test 2 / 10 min. Reply-To set as a raw header to avoid the reply_to/replyTo naming variance. Honeypot hits return fake success. All /api/* responses carry X-Robots-Tag: noindex.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Booking moves to Calendly (35-minute calls)
- bookingUrl now points at calendly.com/darelekan46/35min
- /book page copy updated (35 minutes, Calendly wording)
- Privacy policy processor entry: Google Calendar replaced with Calendly
- Documentation + services spreadsheet regenerated to match

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018A5h36uWK4kcZoHCyNmetT
</commit_message>
<xml_diff>
--- a/docs/dareomotosho-services.xlsx
+++ b/docs/dareomotosho-services.xlsx
@@ -651,7 +651,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Google Calendar appointment schedule</t>
+          <t>Calendly</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -661,27 +661,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The /book page links to a Google Calendar appointment-scheduling page for mentorship/advisory calls</t>
+          <t>The /book page links to a Calendly scheduling page (35-minute calls) for mentorship/advisory</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free tier</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>bookingUrl in lib/site.ts</t>
+          <t>bookingUrl in lib/site.ts (calendly.com/darelekan46/35min)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>calendar.google.com</t>
+          <t>calendly.com dashboard</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Active. Data entered on Google's page is processed by Google (listed in the privacy policy).</t>
+          <t>Active since July 2026, replacing the earlier Google Calendar appointment page. Data entered on Calendly's page is processed by Calendly (listed in the privacy policy).</t>
         </is>
       </c>
     </row>

</xml_diff>